<commit_message>
update to newest chargingstation excel format + update data generic
</commit_message>
<xml_diff>
--- a/data_ProjectTemplate/Chargingstations_ProjectTemplate.xlsx
+++ b/data_ProjectTemplate/Chargingstations_ProjectTemplate.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\AteHe\Desktop\Modellen\Zero_ProjectTemplate\data_ProjectTemplate\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\AteHe\Desktop\Modellen\LUX_ProjectTemplate\data_ProjectTemplate\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CFC6E8C5-A1C7-4E7B-9FCC-0FDCFA03AA1D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CB4DE3F4-9435-4F14-8A09-C9CCF64D576E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2470" yWindow="2230" windowWidth="19200" windowHeight="11180" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="chargingstations" sheetId="2" r:id="rId1"/>
@@ -343,58 +343,32 @@
         </r>
       </text>
     </comment>
-    <comment ref="M1" authorId="0" shapeId="0" xr:uid="{EB6B098B-F5D1-4CBB-AD9A-150B40B161C6}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Luc Sol:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">
-Boolean (mandatory)
-TRUE if it is a charging centre, FALSE if it is a single charging pole</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="N1" authorId="0" shapeId="0" xr:uid="{755A9DE9-FDE3-460A-AB21-427D625FE514}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Luc Sol:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">
-String (optional)
-e.g. cs_0, cs_1
-If empty will look at vehicle_type to generate a profile</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="O1" authorId="0" shapeId="0" xr:uid="{6238DDF5-7C28-4646-8212-258F9F5A9602}">
+    <comment ref="M1" authorId="0" shapeId="0" xr:uid="{755A9DE9-FDE3-460A-AB21-427D625FE514}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Luc Sol:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+boolean (optional)
+If true, charging sessions will be used instead of J_EAEV</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="N1" authorId="0" shapeId="0" xr:uid="{6238DDF5-7C28-4646-8212-258F9F5A9602}">
       <text>
         <r>
           <rPr>
@@ -417,11 +391,11 @@
 String (optional)
 Choose from options:
 CAR, VAN, TRUCK
-Will be ignored if there is profile_data</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="P1" authorId="0" shapeId="0" xr:uid="{07B4133C-8A45-4C3F-B6FC-951506A541F8}">
+</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="O1" authorId="0" shapeId="0" xr:uid="{07B4133C-8A45-4C3F-B6FC-951506A541F8}">
       <text>
         <r>
           <rPr>
@@ -442,38 +416,35 @@
           </rPr>
           <t xml:space="preserve">
 int (optional)
-if is_charging_centre is FALSE this field is ignored and assumed to be 1.
-if there is profile data this field is also ignored</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="Q1" authorId="0" shapeId="0" xr:uid="{AB961B2C-C3E7-4C36-81D0-93E84BEF4C55}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Luc Sol:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">
-double (optional)
-If empty looks at number_of_chargers and vehicle_type.
-if there is profile data this field is ignored</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="R1" authorId="0" shapeId="0" xr:uid="{9910EB31-5FE2-4A9E-AA0B-50E7F5AFACBE}">
+</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="P1" authorId="0" shapeId="0" xr:uid="{AB961B2C-C3E7-4C36-81D0-93E84BEF4C55}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Luc Sol:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+double (optional)</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="Q1" authorId="0" shapeId="0" xr:uid="{9910EB31-5FE2-4A9E-AA0B-50E7F5AFACBE}">
       <text>
         <r>
           <rPr>
@@ -498,7 +469,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="S1" authorId="0" shapeId="0" xr:uid="{7BEDD647-FF3D-4F8D-9179-27813356AD75}">
+    <comment ref="R1" authorId="0" shapeId="0" xr:uid="{7BEDD647-FF3D-4F8D-9179-27813356AD75}">
       <text>
         <r>
           <rPr>
@@ -523,7 +494,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="T1" authorId="0" shapeId="0" xr:uid="{C4B4D0C3-8439-4A64-B20C-03D562CA2B4E}">
+    <comment ref="S1" authorId="0" shapeId="0" xr:uid="{C4B4D0C3-8439-4A64-B20C-03D562CA2B4E}">
       <text>
         <r>
           <rPr>
@@ -554,7 +525,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
   <si>
     <t>polygon</t>
   </si>
@@ -565,21 +536,9 @@
     <t>latitude</t>
   </si>
   <si>
-    <t>power_per_charger_kw</t>
-  </si>
-  <si>
-    <t>number_of_chargers</t>
-  </si>
-  <si>
     <t>vehicle_type</t>
   </si>
   <si>
-    <t>profile_data</t>
-  </si>
-  <si>
-    <t>is_charging_centre</t>
-  </si>
-  <si>
     <t>connection_capacity_kw</t>
   </si>
   <si>
@@ -614,6 +573,15 @@
   </si>
   <si>
     <t>gridnode_id</t>
+  </si>
+  <si>
+    <t>uses_charging_sessions</t>
+  </si>
+  <si>
+    <t>power_per_socket_kw</t>
+  </si>
+  <si>
+    <t>number_of_sockets</t>
   </si>
 </sst>
 </file>
@@ -685,7 +653,7 @@
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Standaard" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -963,90 +931,86 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DD248F3B-E9BA-4D88-9344-99B35CA3C271}">
-  <dimension ref="A1:T1"/>
+  <dimension ref="A1:S1"/>
   <sheetFormatPr defaultColWidth="14.81640625" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="5.26953125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="20.7265625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10.7265625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="13.81640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11.81640625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.26953125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.1796875" customWidth="1"/>
-    <col min="9" max="9" width="6.6328125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="7.54296875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="5.08984375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="8.26953125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="8.7265625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.36328125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.6328125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.36328125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13.90625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="9.90625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="3.6328125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="10.81640625" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="12.54296875" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="21.81640625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="17" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="11.26953125" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="15" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="18.54296875" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="21.26953125" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="7.54296875" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="9.1796875" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="7.7265625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="21.36328125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="20.6328125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="11.1796875" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="18.453125" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="20.81640625" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="7.1796875" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="8.6328125" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="7.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="O1" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="P1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="G1" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="H1" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="I1" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="K1" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="L1" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="M1" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="N1" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="O1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="P1" s="1" t="s">
-        <v>4</v>
-      </c>
       <c r="Q1" s="1" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="R1" s="1" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="S1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="T1" s="1" t="s">
         <v>0</v>
       </c>
     </row>

</xml_diff>